<commit_message>
Update dashboard data, price tracking results, and add new utility scripts
</commit_message>
<xml_diff>
--- a/mapping_review.xlsx
+++ b/mapping_review.xlsx
@@ -28,13 +28,13 @@
     <t>Reason</t>
   </si>
   <si>
-    <t>ACER NITRO V Core I5 RTX 2050</t>
-  </si>
-  <si>
-    <t>Acer Chromebook Plus 515 Intel Core i3 1215U Nvidia GeForce RTX 2050</t>
-  </si>
-  <si>
-    <t>product_line_mismatch</t>
+    <t>SAMSUNG GALAXY BOOK Core 7 GMA</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy Book4 Pro OLED Intel Core Ultra 5 125H Intel Arc Graphics</t>
+  </si>
+  <si>
+    <t>product_line_mismatch,cpu_tier_mismatch</t>
   </si>
 </sst>
 </file>

</xml_diff>